<commit_message>
feat(vlc): implement VLC RTSP source creation and update Player component
</commit_message>
<xml_diff>
--- a/docs/rtsp-ptz-latency-results.xlsx
+++ b/docs/rtsp-ptz-latency-results.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Metric guide'!$A$1:$H$16</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Results!$A$1:$H$7</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Results!$A$1:$H$19</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="50">
   <si>
     <t xml:space="preserve">Change</t>
   </si>
@@ -91,6 +91,54 @@
   </si>
   <si>
     <t xml:space="preserve">00:02,84</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vlc-tcp-500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:01,06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:00,68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:02,36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android | TCP | cache=500 ms | hardware decoding=auto, not forced | channel=Sub | observation=</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:01,15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:00,73</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:01,75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:00,78</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:02,51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:01,11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:00,81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:01,53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:00,95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:01,48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:00,61</t>
   </si>
   <si>
     <t xml:space="preserve">Metric</t>
@@ -137,11 +185,12 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -171,6 +220,11 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="4">
@@ -242,12 +296,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -268,6 +326,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -495,179 +557,479 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="35"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="5" t="s">
+      <c r="E2" s="5"/>
+      <c r="F2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="4"/>
+      <c r="H2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="5" t="s">
+      <c r="E3" s="7"/>
+      <c r="F3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="6"/>
+      <c r="H3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="5" t="s">
+      <c r="E4" s="5"/>
+      <c r="F4" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="4"/>
+      <c r="H4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="5" t="s">
+      <c r="E5" s="7"/>
+      <c r="F5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="6"/>
+      <c r="H5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="5" t="s">
+      <c r="E6" s="5"/>
+      <c r="F6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="4"/>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="5" t="s">
+      <c r="E7" s="7"/>
+      <c r="F7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="6"/>
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="6"/>
+      <c r="F9" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>vlc-tcp-300</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Wi-Fi</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Android | TCP | cache=300 ms | hardware decoding=auto, not forced | channel=Sub | observation=</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>vlc-tcp-300</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Wi-Fi</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Android | TCP | cache=300 ms | hardware decoding=auto, not forced | channel=Sub | observation=</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>vlc-tcp-300</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Wi-Fi</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Android | TCP | cache=300 ms | hardware decoding=auto, not forced | channel=Sub | observation=</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>vlc-tcp-300</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Wi-Fi</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Android | TCP | cache=300 ms | hardware decoding=auto, not forced | channel=Sub | observation=</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>vlc-tcp-300</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Wi-Fi</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Android | TCP | cache=300 ms | hardware decoding=auto, not forced | channel=Sub | observation=</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>vlc-tcp-300</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Wi-Fi</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Android | TCP | cache=300 ms | hardware decoding=auto, not forced | channel=Sub | observation=</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
+  <autoFilter ref="A1:H19"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -687,80 +1049,80 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="100"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>23</v>
+      <c r="A1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>24</v>
+      <c r="B2" s="5" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>25</v>
+      <c r="B3" s="7" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>26</v>
+      <c r="B4" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>27</v>
+      <c r="B5" s="7" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>28</v>
+      <c r="B6" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>30</v>
+      <c r="A7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>32</v>
+      <c r="A8" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>33</v>
+      <c r="B9" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>